<commit_message>
Versión 1.1 — Informes de orientación, columnas UEO/ERG y mejoras
Añade soporte para la hoja «Informes» (barreras/fortalezas, necesidades,
justificación), vinculada por NIA con selección del más reciente. Nuevas
columnas Activada UEO?, Aut. contactar ERG y Contactado ERG con chips de
estado. Fichas mínimas automáticas para NIAs solo en Informes, con toggle
para mostrar/ocultar fichas pendientes de completar.

Mejoras: símbolo ¶ como salto de línea, extracción de NIA tolerante entre
hojas, filtro de Curso Académico que ya no oculta alumnos sin actuaciones,
e impresión compacta del informe individual.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo.xlsx
+++ b/demo.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Ficha" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Informes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2153,7 +2154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T16"/>
+  <dimension ref="A1:W16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2257,6 +2258,21 @@
           <t>Campo Abierto</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Activada UEO?</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Autorización para Contactar ERG?</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Contactado ERG?</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2355,6 +2371,21 @@
       <c r="T2" t="inlineStr">
         <is>
           <t>Necesita refuerzo en autocontrol durante las clases colectivas.</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -2447,6 +2478,21 @@
       <c r="T3" t="inlineStr">
         <is>
           <t>Pendiente informe del logopeda externo.</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2529,6 +2575,21 @@
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2621,6 +2682,21 @@
           <t>Caso cerrado tras adaptación satisfactoria al grupo.</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2719,6 +2795,21 @@
       <c r="T6" t="inlineStr">
         <is>
           <t>Episodios de bloqueo en exámenes. Coordinación con tutora externa.</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
         </is>
       </c>
     </row>
@@ -2797,6 +2888,21 @@
           <t>Programa de enriquecimiento curricular en colaboración con su instituto.</t>
         </is>
       </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2891,6 +2997,21 @@
       <c r="T8" t="inlineStr">
         <is>
           <t>Pendiente cita con psicóloga externa.</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2973,6 +3094,21 @@
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3073,6 +3209,21 @@
           <t>Adaptación de partituras y apoyo emocional continuado.</t>
         </is>
       </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3167,6 +3318,21 @@
       <c r="T11" t="inlineStr">
         <is>
           <t>Preparando pruebas de acceso al Superior.</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -3253,6 +3419,21 @@
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3345,6 +3526,21 @@
           <t>En seguimiento por su tutor del centro de referencia.</t>
         </is>
       </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3439,6 +3635,21 @@
       <c r="T14" t="inlineStr">
         <is>
           <t>Primera matriculación; integración favorable.</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -3505,6 +3716,21 @@
           <t>Caso cerrado al finalizar enseñanzas profesionales.</t>
         </is>
       </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3593,6 +3819,423 @@
           <t>Adaptaciones metodológicas en la clase colectiva. Coordinación con orientadora del IES.</t>
         </is>
       </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>NIA</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Fecha Informe</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Barreras Acceso</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Fortalezas Acceso</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Barreras Participación</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Fortalezas Participación</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Barreras Aprendizaje</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Fortalezas Aprendizaje</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Necesidades específicas de apoyo educativo</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Justificación y orientaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>10001</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>45945</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dificultad para mantener la atención durante sesiones largas.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Alta motivación hacia la música y buena relación con sus iguales.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Tiende a aislarse en actividades grupales cuando se siente insegura.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Participación activa cuando se le asigna un rol claro.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Bajo rendimiento en lectura de partituras a primera vista.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Excelente oído y capacidad memorística para repertorio.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Alumna con TDAH que necesita adaptaciones en la gestión del tiempo, descansos pautados y refuerzo de la lectura musical.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Se recomienda fragmentar las tareas, usar señales visuales y coordinar con la tutora del IES para mantener las mismas estrategias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>10005</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>45981</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Crisis de ansiedad ante evaluaciones formales.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Capacidad técnica adecuada al nivel cuando no hay presión externa.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Tendencia al bloqueo en audiciones y clases magistrales.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Buena interacción con compañeros/as en ensayos de cámara.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Dificultad para generalizar lo aprendido a contextos nuevos.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Creatividad destacable en improvisación y composición libre.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Alumna con TDAH y ansiedad que requiere adaptación de las condiciones de evaluación, apoyo emocional continuado y coordinación con profesional externo.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Se aconseja permitir evaluaciones en entorno controlado, avisar con antelación de las audiciones y mantener comunicación regular con la familia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>10005</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>46063</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Persisten las crisis de ansiedad, aunque se han reducido en frecuencia.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mejora notable en la gestión de la frustración y en la relación con el profesorado.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Evita participar voluntariamente en audiciones.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Participa activamente en pequeño grupo; ha mejorado el trabajo cooperativo.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Lectura a primera vista aún por debajo del nivel esperado.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Rendimiento técnico bueno; musicalidad e interpretación expresiva destacadas.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Se mantienen las necesidades del primer informe. Se añade la necesidad de un plan gradual de exposición a situaciones de interpretación pública.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Continuar con el protocolo de evaluación adaptada. Iniciar exposición progresiva a audiciones (primero en grupo, luego individual). Coordinación trimestral con la psicóloga externa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>10009</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>45996</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Material escrito convencional dificulta el acceso a la información musical.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Excelente capacidad auditiva y de imitación.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Se retrae cuando debe leer en voz alta o seguir indicaciones escritas en clase.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Compañerismo y disposición a ayudar a otros.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Lentitud en la lectura de partituras y dificultad con la nomenclatura convencional.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Gran sensibilidad interpretativa y buena respuesta a metodologías prácticas.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Alumna con dislexia y ansiedad asociada que necesita materiales adaptados (tipografía, espaciado, colores) y metodología centrada en lo auditivo-práctico.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Proporcionar partituras con tipografía OpenDyslexic, ampliar los plazos de entrega y priorizar la evaluación práctica sobre la escrita.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>10015</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>46040</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Dificultad para interpretar instrucciones ambiguas o implícitas.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Constancia, disciplina y alto interés por la música.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Necesita estructura y anticipación para participar en actividades no rutinarias.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Una vez integrada, participa con entusiasmo y aporta ideas originales.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Puede perder el hilo en sesiones con múltiples cambios de actividad.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Excelente capacidad de concentración cuando la tarea es clara y estructurada.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Alumna con TEA leve que requiere anticipación de cambios, instrucciones explícitas y material visual de apoyo.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Usar apoyos visuales (horarios, secuencias), anticipar los cambios de actividad con al menos 5 minutos, y coordinar con la orientadora del IES las adaptaciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>10099</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>46073</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Dificultad de acceso al transporte adaptado.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Familia implicada y alto interés del alumno/a.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Participación limitada en actividades fuera del aula habitual.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Buena relación con el grupo clase.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Rendimiento irregular por absentismo justificado.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Capacidad de trabajo autónomo cuando dispone de material adaptado.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Alumno/a con necesidades de apoyo por situación sociofamiliar compleja. ¶ Requiere flexibilización horaria y seguimiento de asistencia.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Coordinar con servicios sociales. ¶ Permitir asistencia flexible y facilitar materiales para trabajo autónomo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>10002</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>46082</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Lectura lenta de textos escritos y nomenclatura musical.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Buena comprensión oral y capacidad de razonamiento musical.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Tiende a inhibirse en actividades que implican lectura pública.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Participación activa en debates y actividades orales.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Errores frecuentes en la escritura de dictados musicales.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Memoria auditiva excelente; reproduce fragmentos complejos tras escucharlos.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Alumno con dislexia que necesita adaptaciones en la presentación del material escrito y evaluación preferentemente oral o práctica.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Ampliar tiempos de lectura, usar partituras con mayor espaciado y facilitar grabaciones de audio como complemento al material escrito.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>